<commit_message>
Update prompt checklist live status
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -433,6 +433,7 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -461,6 +462,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Live/Gepusht</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -624,6 +630,11 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>Dashboard decision-supportlaag aangescherpt en gevalideerd; managementread, productspecifieke duiding en tests opgeleverd.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Gepusht (niet live)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document dashboard live validation
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -629,12 +629,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dashboard decision-supportlaag aangescherpt en gevalideerd; managementread, productspecifieke duiding en tests opgeleverd.</t>
+          <t>Dashboard decision-supportlaag aangescherpt en gevalideerd; managementread, productspecifieke duiding en tests opgeleverd. Publieke productiechecks uitgevoerd; volledige campaign-validatie vereist ingelogde live sessie.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Main gepusht; livecheck open</t>
+          <t>Main gepusht; publieke livechecks gedaan; auth-validatie open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update prompt checklist after ExitScan implementation
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Opgeleverd: EXITSCAN_PRODUCT_REVIEW_AND_TEST_PLAN.md plus ExitScan alignment, parity- en smoke-tests</t>
+          <t>Opgeleverd: EXITSCAN_PRODUCT_REVIEW_AND_TEST_PLAN.md plus ExitScan alignment, parity- en smoke-tests; gecommit en gepusht op codex/dashboard-decision-support</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sharpen RetentieScan positioning and methodology
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -531,12 +531,15 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>46126</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>RETENTIESCAN_PRODUCT_REVIEW_AND_TEST_PLAN.md toegevoegd; RetentieScan-copy, methodologie en tests aangescherpt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add prompt system and live test planning assets
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,7 +489,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Opgeleverd: EXITSCAN_PRODUCT_REVIEW_AND_TEST_PLAN.md plus ExitScan alignment, parity- en smoke-tests; gecommit en gepusht op codex/dashboard-decision-support</t>
+          <t>Opgeleverd: EXITSCAN_PRODUCT_REVIEW_AND_TEST_PLAN.md plus ExitScan alignment, parity- en smoke-tests; wordt via main live meegenomen.</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Live via main (na merge)</t>
         </is>
       </c>
     </row>
@@ -514,7 +519,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>EXITSCAN_LIVE_TEST_PLAN.md opgeleverd en aangevuld met eerste live checks en blockers voor ExitScan.</t>
+          <t>EXITSCAN_LIVE_TEST_PLAN.md opgeleverd; dit is een live testplan en geen deploybaar productonderdeel.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Gepusht (plan only, n.v.t. live)</t>
         </is>
       </c>
     </row>
@@ -539,7 +549,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>RETENTIESCAN_PRODUCT_REVIEW_AND_TEST_PLAN.md toegevoegd; RetentieScan-copy, methodologie en tests aangescherpt.</t>
+          <t>RETENTIESCAN_PRODUCT_REVIEW_AND_TEST_PLAN.md toegevoegd; RetentieScan-copy, methodologie en tests aangescherpt en wordt via main live meegenomen.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Live via main (na merge)</t>
         </is>
       </c>
     </row>
@@ -625,19 +640,17 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
+      <c r="D8" s="2" t="n">
+        <v>46126</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dashboard decision-supportlaag aangescherpt en gevalideerd; managementread, productspecifieke duiding en tests opgeleverd.</t>
+          <t>Dashboard decision-supportlaag aangescherpt en gevalideerd; managementread, productspecifieke duiding en tests worden via main live meegenomen.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Gepusht (niet live)</t>
+          <t>Live via main (na merge)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Execute ExitScan live test plan
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -54,9 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -520,7 +523,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>EXITSCAN_LIVE_TEST_PLAN.md opgeleverd; dit is een live testplan en geen deploybaar productonderdeel.</t>
+          <t>EXITSCAN_LIVE_TEST_PLAN.md live doorlopen met fixture-org, role-based dashboardchecks, survey-statevalidatie en blockers op open survey, PDF en reminder.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -574,16 +577,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>46126</v>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>RETENTIESCAN_LIVE_TEST_PLAN.md opgeleverd; live testplan voor site, CTA, auth, survey, dashboard, trendlaag, segmentlaag en rapportdownload.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Gepusht (plan only, n.v.t. live)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -601,13 +610,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -625,13 +632,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -681,13 +686,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -705,13 +708,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -729,13 +730,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -753,13 +752,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -777,13 +774,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -801,13 +796,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -825,13 +818,11 @@
           <t>Niet voldaan</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Document ExitScan live deployment validation
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -523,12 +523,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>EXITSCAN_LIVE_TEST_PLAN.md live doorlopen met fixture-org, role-based dashboardchecks, survey-statevalidatie en blockers op open survey, PDF en reminder.</t>
+          <t>EXITSCAN_LIVE_TEST_PLAN.md live doorlopen, fixes gedeployed op main en hergevalideerd voor forgot-password, survey, PDF en reminder.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Gepusht (plan only, n.v.t. live)</t>
+          <t>Live op main; Supabase RPC toegepast en kernfixes hergevalideerd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document RetentieScan live test end state
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,7 +577,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Voldaan</t>
+          <t>Niet voldaan</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -585,12 +585,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>RETENTIESCAN_LIVE_TEST_PLAN.md opgeleverd; live testplan voor site, CTA, auth, survey, dashboard, trendlaag, segmentlaag en rapportdownload.</t>
+          <t>RETENTIESCAN_LIVE_TEST_PLAN.md live uitgevoerd en bijgewerkt als source of truth. Survey open-token, invalid-token en forgot-password zijn live hersteld; admin invite-route en reminder-UI zijn ook live gerepareerd. Resterend open: contact- en reminder-mails leveren nog niet af door externe Resend-configuratie (send.verisight.nl niet geverifieerd).</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Gepusht (plan only, n.v.t. live)</t>
+          <t>Deels live hersteld; repo-fixes gepusht op main, maar e-maillevering blijft geblokkeerd door Resend-domeinconfig.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Archive completed plan docs and track retention sharpening plan
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -585,12 +585,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>RETENTIESCAN_LIVE_TEST_PLAN.md live uitgevoerd en bijgewerkt als source of truth. Survey open-token, invalid-token en forgot-password zijn live hersteld; admin invite-route en reminder-UI zijn ook live gerepareerd. Resterend open: contact- en reminder-mails leveren nog niet af door externe Resend-configuratie (send.verisight.nl niet geverifieerd).</t>
+          <t>RETENTIESCAN_LIVE_TEST_PLAN.md live uitgevoerd en bijgewerkt als source of truth. Survey open-token, invalid-token, forgot-password, admin invite-route en reminder-UI zijn live hersteld. Note: reminder- en contactmail leveren nog niet af door externe Resend-configuratie (send.verisight.nl niet geverifieerd); dit staat als aparte ops-note buiten de repo-uitwerking.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Deels live hersteld; repo-fixes gepusht op main, maar e-maillevering blijft geblokkeerd door Resend-domeinconfig.</t>
+          <t>Voldaan; repo- en livewijzigingen doorgevoerd op main. Externe ops-note: Resend-domeinverificatie nog open voor maillevering.</t>
         </is>
       </c>
     </row>
@@ -607,12 +607,20 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>46126</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>RETENTIESCAN_PRODUCT_SHARPENING_PLAN.md actief toegevoegd als source-of-truth plan voor de aanscherpingsfase.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Live via main (plan only)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sharpen RetentieScan positioning and report language
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -615,12 +615,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>RETENTIESCAN_PRODUCT_SHARPENING_PLAN.md actief toegevoegd als source-of-truth plan voor de aanscherpingsfase.</t>
+          <t>RETENTIESCAN_PRODUCT_SHARPENING_PLAN.md uitgevoerd; RetentieScan-copy, survey-intro, dashboardduiding, rapporttaal, paritychecks en regressietests aangescherpt en gevalideerd met tests, lint en build.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Live via main (plan only)</t>
+          <t>Live via main</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement RetentieScan v1.1 validation framework
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -56,10 +57,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -637,12 +639,20 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>46126</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>RETENTIESCAN_V1_1_VALIDATION_PLAN.md uitgevoerd; evidence/claims-model, measurement/interpretation-QA en real-data/acceptance docs toegevoegd; validatiescripts kregen dataset-provenance guardrails en het planbestand is milestone-voor-milestone bijgewerkt.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; backend- en frontend-validatie groen.</t>
         </is>
       </c>
     </row>
@@ -829,6 +839,226 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>Werk deze rij bij na uitvoering van de prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Nu. Focus op flow van websitebezoek naar demo, intake, livegang en rapportgebruik.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>METHOD_AND_TRUST_SYSTEM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>METHOD_AND_TRUST_SYSTEM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Nu. Verduidelijk methodiek, AVG, interpretatiegrenzen en commerci?le geloofwaardigheid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Nu. Richt onboarding, livegang en eerste managementgebruik beter in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Daarna. Maak demo-omgeving, voorbeeldcampagnes en demo-scripts schaalbaar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Daarna. Breng vaste producttaal over site, dashboard, rapport en sales samen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>REPORT_TO_ACTION_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>REPORT_TO_ACTION_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Daarna. Maak de stap van rapport naar concrete managementactie expliciet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Scherp de samenhang tussen ExitScan, RetentieScan en toekomstige producten aan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerci?le bewijsvoering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CONTENT_OPERATING_SYSTEM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CONTENT_OPERATING_SYSTEM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Laat site, SEO, cases en thought leadership ??n systeem vormen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>OPS_AND_DELIVERY_SYSTEM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>OPS_AND_DELIVERY_SYSTEM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Stroomlijn delivery van sales handoff tot rapportoplevering en nazorg.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update prompt checklist ordering and add planning backlog
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -439,32 +439,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Prompt File</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Live/Gepusht</t>
         </is>
@@ -582,7 +582,7 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>46126</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -612,7 +612,7 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>46126</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -629,12 +629,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>RETENTIESCAN_V1_1_VALIDATION_PLANMODE_PROMPT.md</t>
+          <t>DASHBOARD_DECISION_SUPPORT_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RETENTIESCAN_V1_1_VALIDATION_PLAN.md</t>
+          <t>DASHBOARD_DECISION_SUPPORT_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -642,29 +642,31 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n">
-        <v>46126</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>RETENTIESCAN_V1_1_VALIDATION_PLAN.md uitgevoerd; evidence/claims-model, measurement/interpretation-QA en real-data/acceptance docs toegevoegd; validatiescripts kregen dataset-provenance guardrails en het planbestand is milestone-voor-milestone bijgewerkt.</t>
+          <t>Dashboard decision-supportlaag aangescherpt en gevalideerd; managementread, productspecifieke duiding en tests worden via main live meegenomen.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; backend- en frontend-validatie groen.</t>
+          <t>Live via main</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DASHBOARD_DECISION_SUPPORT_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>RETENTIESCAN_V1_1_VALIDATION_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DASHBOARD_DECISION_SUPPORT_PROGRAM_PLAN.md</t>
+          <t>RETENTIESCAN_V1_1_VALIDATION_PLAN.md</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -672,19 +674,17 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-04-14</t>
-        </is>
+      <c r="D8" s="3" t="n">
+        <v>46126</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dashboard decision-supportlaag aangescherpt en gevalideerd; managementread, productspecifieke duiding en tests worden via main live meegenomen.</t>
+          <t>RETENTIESCAN_V1_1_VALIDATION_PLAN.md uitgevoerd; evidence/claims-model, measurement/interpretation-QA en real-data/acceptance docs toegevoegd; validatiescripts kregen dataset-provenance guardrails en het planbestand is milestone-voor-milestone bijgewerkt.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Live via main</t>
+          <t>Uitgevoerd in repo; backend- en frontend-validatie groen.</t>
         </is>
       </c>
     </row>
@@ -713,12 +713,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>WEBSITE_REDESIGN_AND_FLOW_PLANMODE_PROMPT.md</t>
+          <t>REPORT_VISUAL_AND_COMMERCIAL_UPLIFT_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md</t>
+          <t>REPORT_VISUAL_AND_COMMERCIAL_UPLIFT_PLAN.md</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -728,19 +728,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Nu. Maak rapporten visueler, commerci?ler, sterker voor MT en minder stoffig of theoretisch.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SEO_CONVERSION_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>MANAGEMENT_ACTIONABILITY_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SEO_CONVERSION_PROGRAM_PLAN.md</t>
+          <t>MANAGEMENT_ACTIONABILITY_PLAN.md</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -750,19 +750,19 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Nu. Maak de stap van inzicht naar managementvraag, besluit en actie explicieter.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PRICING_AND_PACKAGING_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>BOARDROOM_READINESS_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PRICING_AND_PACKAGING_PROGRAM_PLAN.md</t>
+          <t>BOARDROOM_READINESS_PLAN.md</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -772,19 +772,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Nu. Maak output geschikter voor directie, bestuur en besluitvorming op hoog niveau.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SALES_ENABLEMENT_SYSTEM_PLANMODE_PROMPT.md</t>
+          <t>METHOD_AND_TRUST_SYSTEM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SALES_ENABLEMENT_SYSTEM_PLAN.md</t>
+          <t>METHOD_AND_TRUST_SYSTEM_PLAN.md</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -794,19 +794,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Nu. Verduidelijk methodiek, AVG, interpretatiegrenzen en commerci?le geloofwaardigheid.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>IMPLEMENTATION_READINESS_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>TRUST_SIGNAL_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IMPLEMENTATION_READINESS_PROGRAM_PLAN.md</t>
+          <t>TRUST_SIGNAL_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -816,19 +816,19 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Nu. Versterk zichtbare betrouwbaarheid via methodiek, privacy, professionaliteit en legitimiteit.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PILOT_AND_EARLY_CUSTOMER_LEARNING_SYSTEM_PLANMODE_PROMPT.md</t>
+          <t>FOUNDER_LED_SALES_NARRATIVE_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PILOT_AND_EARLY_CUSTOMER_LEARNING_SYSTEM_PLAN.md</t>
+          <t>FOUNDER_LED_SALES_NARRATIVE_PLAN.md</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -838,19 +838,19 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Nu. Scherp het founder-verhaal, bezwaarbehandeling en productnarratief aan.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLANMODE_PROMPT.md</t>
+          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLAN.md</t>
+          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLAN.md</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -860,19 +860,19 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Focus op flow van websitebezoek naar demo, intake, livegang en rapportgebruik.</t>
+          <t>Aanbevolen prioriteit: Daarna. Breng vaste producttaal over site, dashboard, rapport en sales samen.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>METHOD_AND_TRUST_SYSTEM_PLANMODE_PROMPT.md</t>
+          <t>SALES_ENABLEMENT_SYSTEM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>METHOD_AND_TRUST_SYSTEM_PLAN.md</t>
+          <t>SALES_ENABLEMENT_SYSTEM_PLAN.md</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -882,19 +882,19 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Verduidelijk methodiek, AVG, interpretatiegrenzen en commerci?le geloofwaardigheid.</t>
+          <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>PRICING_AND_PACKAGING_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLAN.md</t>
+          <t>PRICING_AND_PACKAGING_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -904,19 +904,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Richt onboarding, livegang en eerste managementgebruik beter in.</t>
+          <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>SAMPLE_OUTPUT_AND_SHOWCASE_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLAN.md</t>
+          <t>SAMPLE_OUTPUT_AND_SHOWCASE_PLAN.md</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -926,19 +926,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Maak demo-omgeving, voorbeeldcampagnes en demo-scripts schaalbaar.</t>
+          <t>Aanbevolen prioriteit: Daarna. Bouw sterke voorbeeldrapporten, demo-output en showcase-assets.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLANMODE_PROMPT.md</t>
+          <t>WEBSITE_REDESIGN_AND_FLOW_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLAN.md</t>
+          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -948,19 +948,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Breng vaste producttaal over site, dashboard, rapport en sales samen.</t>
+          <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>REPORT_TO_ACTION_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>SEO_CONVERSION_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>REPORT_TO_ACTION_PROGRAM_PLAN.md</t>
+          <t>SEO_CONVERSION_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -970,19 +970,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Maak de stap van rapport naar concrete managementactie expliciet.</t>
+          <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md</t>
+          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLAN.md</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -992,19 +992,19 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Scherp de samenhang tussen ExitScan, RetentieScan en toekomstige producten aan.</t>
+          <t>Aanbevolen prioriteit: Nu. Focus op flow van websitebezoek naar demo, intake, livegang en rapportgebruik.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md</t>
+          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1014,19 +1014,19 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerci?le bewijsvoering.</t>
+          <t>Aanbevolen prioriteit: Nu. Richt onboarding, livegang en eerste managementgebruik beter in.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CONTENT_OPERATING_SYSTEM_PLANMODE_PROMPT.md</t>
+          <t>IMPLEMENTATION_READINESS_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CONTENT_OPERATING_SYSTEM_PLAN.md</t>
+          <t>IMPLEMENTATION_READINESS_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1036,29 +1036,161 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Laat site, SEO, cases en thought leadership ??n systeem vormen.</t>
+          <t>Werk deze rij bij na uitvoering van de prompt</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>REPORT_TO_ACTION_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>REPORT_TO_ACTION_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Daarna. Maak de stap van rapport naar concrete managementactie expliciet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PILOT_AND_EARLY_CUSTOMER_LEARNING_SYSTEM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PILOT_AND_EARLY_CUSTOMER_LEARNING_SYSTEM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Werk deze rij bij na uitvoering van de prompt</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>OPS_AND_DELIVERY_SYSTEM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>OPS_AND_DELIVERY_SYSTEM_PLAN.md</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Niet voldaan</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>Aanbevolen prioriteit: Later. Stroomlijn delivery van sales handoff tot rapportoplevering en nazorg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Daarna. Maak demo-omgeving, voorbeeldcampagnes en demo-scripts schaalbaar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Scherp de samenhang tussen ExitScan, RetentieScan en toekomstige producten aan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerci?le bewijsvoering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CONTENT_OPERATING_SYSTEM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>CONTENT_OPERATING_SYSTEM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Laat site, SEO, cases en thought leadership ??n systeem vormen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sharpen reporting system parity and report content
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -701,12 +701,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>REPORTING_SYSTEM_SHARPENING_PLAN.md toegevoegd; report-content contracts, productspecifieke managementsamenvattingen, signal-page/hypothese/vervolgstap-copy en paritytests voor backend/frontend aangescherpt en gevalideerd met pytest, vitest, eslint en Next build.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Live via main</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement report visual and commercial uplift
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -733,12 +733,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Maak rapporten visueler, commerci?ler, sterker voor MT en minder stoffig of theoretisch.</t>
+          <t>REPORT_VISUAL_AND_COMMERCIAL_UPLIFT_PLAN.md uitgevoerd; echte PDF-output kreeg executive shell, highlight cards, trust-notes, productspecifieke themakleuren, preview/report parity, smoke-tests en acceptance-checklist.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Live via main</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align planning system roadmap and prompt inventory
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -777,12 +777,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BOARDROOM_READINESS_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>METHOD_AND_TRUST_SYSTEM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BOARDROOM_READINESS_PLAN.md</t>
+          <t>METHOD_AND_TRUST_SYSTEM_PLAN.md</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -792,19 +792,19 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Maak output geschikter voor directie, bestuur en besluitvorming op hoog niveau.</t>
+          <t>Aanbevolen prioriteit: Nu. Verduidelijk methodiek, AVG, interpretatiegrenzen en commerci?le geloofwaardigheid.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>METHOD_AND_TRUST_SYSTEM_PLANMODE_PROMPT.md</t>
+          <t>TRUST_SIGNAL_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>METHOD_AND_TRUST_SYSTEM_PLAN.md</t>
+          <t>TRUST_SIGNAL_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -814,19 +814,19 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Verduidelijk methodiek, AVG, interpretatiegrenzen en commerci?le geloofwaardigheid.</t>
+          <t>Aanbevolen prioriteit: Nu. Versterk zichtbare betrouwbaarheid via methodiek, privacy, professionaliteit en legitimiteit.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TRUST_SIGNAL_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>BOARDROOM_READINESS_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TRUST_SIGNAL_PROGRAM_PLAN.md</t>
+          <t>BOARDROOM_READINESS_PLAN.md</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Versterk zichtbare betrouwbaarheid via methodiek, privacy, professionaliteit en legitimiteit.</t>
+          <t>Aanbevolen prioriteit: Nu. Maak output geschikter voor directie, bestuur en besluitvorming op hoog niveau.</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Scherp het founder-verhaal, bezwaarbehandeling en productnarratief aan.</t>
+          <t>Aanbevolen prioriteit: Nu. Scherp het founder-verhaal, bezwaren, demo-volgorde en productnarratief aan.</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Daarna. Maak sales-assets en demo-ondersteuning consistent met de aangescherpte propositie.</t>
         </is>
       </c>
     </row>
@@ -924,7 +924,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Daarna. Werk prijslogica, Baseline/Live en packaging commercieel strak uit.</t>
         </is>
       </c>
     </row>
@@ -968,19 +968,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Daarna. Doe website-redesign pas na trust, actionability, packaging en sample output.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SEO_CONVERSION_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SEO_CONVERSION_PROGRAM_PLAN.md</t>
+          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLAN.md</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -990,19 +990,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Daarna. Stem funnel en klantreis af nadat website- en packagingrichting scherper staan.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLANMODE_PROMPT.md</t>
+          <t>SEO_CONVERSION_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLAN.md</t>
+          <t>SEO_CONVERSION_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Focus op flow van websitebezoek naar demo, intake, livegang en rapportgebruik.</t>
+          <t>Aanbevolen prioriteit: Daarna. Optimaliseer SEO en conversie pas na website-redesign en stabiele messaging.</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Richt onboarding, livegang en eerste managementgebruik beter in.</t>
+          <t>Aanbevolen prioriteit: Later. Richt onboarding, livegang en eerste managementgebruik beter in zodra commerci?le basis staat.</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Later. Maak implementation readiness schaalbaar na scherpere commerci?le en websitebasis.</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Maak de stap van rapport naar concrete managementactie expliciet.</t>
+          <t>Aanbevolen prioriteit: Later. Versterk de stap van rapport naar concrete managementactie na de bredere actionability-laag.</t>
         </is>
       </c>
     </row>
@@ -1100,19 +1100,19 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Werk deze rij bij na uitvoering van de prompt</t>
+          <t>Aanbevolen prioriteit: Later. Borg leerloops en pilotfeedback zodra eerste klanttrajecten lopen.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OPS_AND_DELIVERY_SYSTEM_PLANMODE_PROMPT.md</t>
+          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OPS_AND_DELIVERY_SYSTEM_PLAN.md</t>
+          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1122,19 +1122,19 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Stroomlijn delivery van sales handoff tot rapportoplevering en nazorg.</t>
+          <t>Aanbevolen prioriteit: Later. Maak demo-omgeving en voorbeeldcampagnes schaalbaar na sample-output en salesbasis.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>OPS_AND_DELIVERY_SYSTEM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLAN.md</t>
+          <t>OPS_AND_DELIVERY_SYSTEM_PLAN.md</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1144,19 +1144,19 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Maak demo-omgeving, voorbeeldcampagnes en demo-scripts schaalbaar.</t>
+          <t>Aanbevolen prioriteit: Later. Stroomlijn delivery van sales handoff tot rapportoplevering en nazorg.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md</t>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1166,19 +1166,19 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Scherp de samenhang tussen ExitScan, RetentieScan en toekomstige producten aan.</t>
+          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerci?le bewijsvoering na echte pilots.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md</t>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerci?le bewijsvoering.</t>
+          <t>Aanbevolen prioriteit: Later. Scherp de samenhang tussen ExitScan, RetentieScan en toekomstige producten aan.</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Laat site, SEO, cases en thought leadership ??n systeem vormen.</t>
+          <t>Aanbevolen prioriteit: Later. Laat site, SEO, cases en thought leadership pas als systeem groeien na product- en funnelstabiliteit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sharpen management actionability across dashboard and reports
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -765,12 +765,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>46126</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Maak de stap van inzicht naar managementvraag, besluit en actie explicieter.</t>
+          <t>MANAGEMENT_ACTIONABILITY_PLAN.md toegevoegd; ExitScan kreeg besluit- en eigenaarschapsroutes in dashboard en report, RetentieScan-toplaag werd aangescherpt op eerste besluit/eigenaar, action playbooks en focusvragen zijn herbouwd en paritytests zijn groen gevalideerd met pytest, vitest, lint en Next build.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; niet gepusht in deze turn.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync roadmap and prompt checklist status
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -773,12 +773,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MANAGEMENT_ACTIONABILITY_PLAN.md toegevoegd; ExitScan kreeg besluit- en eigenaarschapsroutes in dashboard en report, RetentieScan-toplaag werd aangescherpt op eerste besluit/eigenaar, action playbooks en focusvragen zijn herbouwd en paritytests zijn groen gevalideerd met pytest, vitest, lint en Next build.</t>
+          <t>MANAGEMENT_ACTIONABILITY_PLAN.md uitgevoerd; ExitScan kreeg besluit- en eigenaarschapsroutes in dashboard en report, RetentieScan-toplaag werd aangescherpt op eerste besluit/eigenaar, action playbooks en focusvragen zijn herbouwd en paritytests zijn groen gevalideerd met pytest, vitest, lint en Next build.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; niet gepusht in deze turn.</t>
+          <t>Naar main gepusht op 2026-04-14 (commit 7025245).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add roadmap and checklist sync workflow
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Prompt Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,22 +16,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -57,11 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,14 +418,6 @@
   </sheetPr>
   <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -582,7 +563,7 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="1" t="n">
         <v>46126</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -612,7 +593,7 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="1" t="n">
         <v>46126</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -674,7 +655,7 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" s="1" t="n">
         <v>46126</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -768,7 +749,7 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="1" t="n">
         <v>46126</v>
       </c>
       <c r="E11" t="inlineStr">
@@ -800,7 +781,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Verduidelijk methodiek, AVG, interpretatiegrenzen en commerci?le geloofwaardigheid.</t>
+          <t>Aanbevolen prioriteit: Nu. Verduidelijk methodiek, AVG, interpretatiegrenzen en commerciële geloofwaardigheid.</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1023,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Richt onboarding, livegang en eerste managementgebruik beter in zodra commerci?le basis staat.</t>
+          <t>Aanbevolen prioriteit: Later. Richt onboarding, livegang en eerste managementgebruik beter in zodra commerciële basis staat.</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1045,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Maak implementation readiness schaalbaar na scherpere commerci?le en websitebasis.</t>
+          <t>Aanbevolen prioriteit: Later. Maak implementation readiness schaalbaar na scherpere commerciële en websitebasis.</t>
         </is>
       </c>
     </row>
@@ -1174,7 +1155,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerci?le bewijsvoering na echte pilots.</t>
+          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerciële bewijsvoering na echte pilots.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve contact form delivery diagnostics
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -776,12 +776,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Verduidelijk methodiek, AVG, interpretatiegrenzen en commerciële geloofwaardigheid.</t>
+          <t>METHOD_AND_TRUST_SYSTEM_PLAN.md toegevoegd; methode- en trustcontract vastgezet over reference docs, frontend/backend productdefinities, report trustblokken, marketing- en legalcopy en regressietests. Frontend tests, lint, build en backend parity/smoke/validation tests groen bevestigd.</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; push naar main volgt in deze ronde.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement trust signal program
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; push naar main volgt in deze ronde.</t>
+          <t>Uitgevoerd in repo; gepusht naar main op 2026-04-14.</t>
         </is>
       </c>
     </row>
@@ -808,12 +808,22 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Versterk zichtbare betrouwbaarheid via methodiek, privacy, professionaliteit en legitimiteit.</t>
+          <t>TRUST_SIGNAL_PROGRAM_PLAN.md toegevoegd; buyer-facing trusthub, gedeelde trust-contentlaag, preview/contact/legal uplift en regressietests voor zichtbare trust-signals uitgevoerd en groen bevestigd.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; frontend tests, lint, build en backend paritytests groen bevestigd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement boardroom readiness program
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -813,17 +813,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>TRUST_SIGNAL_PROGRAM_PLAN.md toegevoegd; buyer-facing trusthub, gedeelde trust-contentlaag, preview/contact/legal uplift en regressietests voor zichtbare trust-signals uitgevoerd en groen bevestigd.</t>
+          <t>TRUST_SIGNAL_PROGRAM_PLAN.md toegevoegd; buyer-facing trusthub, gedeelde trust-contentlaag, preview/contact/legal uplift en regressietests voor zichtbare trust-signals uitgevoerd. Trusthub-route /vertrouwen daarna publiek live gezet op www.verisight.nl.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; frontend tests, lint, build en backend paritytests groen bevestigd.</t>
+          <t>Uitgevoerd in repo en live bevestigd; frontend tests, lint, build, backend paritytests en productie smoke checks groen bevestigd.</t>
         </is>
       </c>
     </row>
@@ -840,12 +840,20 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Maak output geschikter voor directie, bestuur en besluitvorming op hoog niveau.</t>
+          <t>BOARDROOM_READINESS_PLAN.md toegevoegd; report- en dashboardcontracten kregen een bestuurlijke handoff, preview/marketing/pricing zijn op dezelfde senior leeslijn gezet, voorbeeldrapporten vernieuwd en parity/smoke-tests groen gevalideerd.</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; pytest, vitest, eslint, Next build en sample-output groen op 2026-04-15. Nog niet gepusht.</t>
         </is>
       </c>
     </row>
@@ -862,12 +870,20 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Nu. Scherp het founder-verhaal, bezwaren, demo-volgorde en productnarratief aan.</t>
+          <t>FOUNDER_LED_SALES_NARRATIVE_PLAN.md toegevoegd; playbook, acceptance checklist, buyer-facing routecopy, preview/boardroom handoff en proposal/pricing-framing vastgelegd.</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; vitest, next build en pytest parity/smoke groen op 2026-04-15.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update boardroom checklist live status
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -848,12 +848,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BOARDROOM_READINESS_PLAN.md toegevoegd; report- en dashboardcontracten kregen een bestuurlijke handoff, preview/marketing/pricing zijn op dezelfde senior leeslijn gezet, voorbeeldrapporten vernieuwd en parity/smoke-tests groen gevalideerd.</t>
+          <t>BOARDROOM_READINESS_PLAN.md toegevoegd; report- en dashboardcontracten kregen een bestuurlijke handoff, preview/marketing/pricing zijn op dezelfde senior leeslijn gezet, voorbeeldrapporten vernieuwd en parity/smoke-tests groen gevalideerd. Publieke marketingcopy live bevestigd op www.verisight.nl en /producten/exitscan.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; pytest, vitest, eslint, Next build en sample-output groen op 2026-04-15. Nog niet gepusht.</t>
+          <t>Naar main gepusht op 2026-04-15; live bevestigd op publieke routes www.verisight.nl en /producten/exitscan. Authenticated dashboard/report-output niet apart live geverifieerd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Confirm founder-led rollout is live
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -878,12 +878,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FOUNDER_LED_SALES_NARRATIVE_PLAN.md toegevoegd; playbook, acceptance checklist, buyer-facing routecopy, preview/boardroom handoff en proposal/pricing-framing vastgelegd.</t>
+          <t>FOUNDER_LED_SALES_NARRATIVE_PLAN.md toegevoegd; playbook, acceptance checklist, buyer-facing routecopy, preview/boardroom handoff en proposal/pricing-framing vastgelegd. Live routes bevestigd op www.verisight.nl.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; vitest, next build en pytest parity/smoke groen op 2026-04-15.</t>
+          <t>Ja: live bevestigd op 2026-04-15 via https://www.verisight.nl, /tarieven en /vertrouwen; founder-led termen zichtbaar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement product terminology system
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -900,12 +900,22 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Breng vaste producttaal over site, dashboard, rapport en sales samen.</t>
+          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLAN.md toegevoegd; canonieke glossary en reviewchecklist vastgelegd, marketing/product/report/survey/sales-termen geharmoniseerd en paritytests, lint en build groen.</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; vitest, pytest, lint en build lokaal groen bevestigd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark terminology plan live in checklist
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -910,12 +910,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLAN.md toegevoegd; canonieke glossary en reviewchecklist vastgelegd, marketing/product/report/survey/sales-termen geharmoniseerd en paritytests, lint en build groen.</t>
+          <t>PRODUCT_TERMINOLOGY_AND_TAXONOMY_SYSTEM_PLAN.md toegevoegd; canonieke glossary en reviewchecklist vastgelegd, marketing/product/report/survey/sales-termen geharmoniseerd en paritytests, lint en build groen; live op main.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; vitest, pytest, lint en build lokaal groen bevestigd.</t>
+          <t>Live via main</t>
         </is>
       </c>
     </row>
@@ -932,12 +932,20 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Maak sales-assets en demo-ondersteuning consistent met de aangescherpte propositie.</t>
+          <t>SALES_ENABLEMENT_SYSTEM_PLAN.md toegevoegd; sales enablement playbook, decision tree, comparison matrix, objection/claims matrix, proposal spines, acceptance checklist en buyer-facing one-pagers toegevoegd. Parity bevestigd via pytest en vitest.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; nog niet gepusht.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update sales enablement checklist status
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -940,12 +940,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>SALES_ENABLEMENT_SYSTEM_PLAN.md toegevoegd; sales enablement playbook, decision tree, comparison matrix, objection/claims matrix, proposal spines, acceptance checklist en buyer-facing one-pagers toegevoegd. Validatie bevestigd via pytest, vitest, eslint en next build.</t>
+          <t>SALES_ENABLEMENT_SYSTEM_PLAN.md toegevoegd; sales enablement playbook, decision tree, comparison matrix, objection/claims matrix, proposal spines, acceptance checklist en buyer-facing one-pagers toegevoegd. Validatie bevestigd via pytest, vitest, eslint en next build. Daarna naar main gepusht.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; nog niet gepusht.</t>
+          <t>Naar main gepusht op 2026-04-15 (aa7ce22); geen aparte publieke livewijziging, alleen repo-assets.</t>
         </is>
       </c>
     </row>
@@ -1172,12 +1172,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OPS_AND_DELIVERY_SYSTEM_PLANMODE_PROMPT.md</t>
+          <t>ASSISTED_TO_SAAS_READINESS_PROGRAM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>OPS_AND_DELIVERY_SYSTEM_PLAN.md</t>
+          <t>ASSISTED_TO_SAAS_READINESS_PROGRAM_PLAN.md</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1187,19 +1187,19 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Stroomlijn delivery van sales handoff tot rapportoplevering en nazorg.</t>
+          <t>Aanbevolen prioriteit: Later. Bepaal wanneer en hoe Verisight van assisted/productized aanbod richting SaaS-readiness mag bewegen.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>CUSTOMER_LIFECYCLE_AND_EXPANSION_MODEL_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md</t>
+          <t>CUSTOMER_LIFECYCLE_AND_EXPANSION_MODEL_PLAN.md</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1209,19 +1209,19 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerciële bewijsvoering na echte pilots.</t>
+          <t>Aanbevolen prioriteit: Later. Werk de route uit van eerste sale naar herhaalgebruik, uitbreiding en productdoorstroom.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLANMODE_PROMPT.md</t>
+          <t>ACCOUNT_AND_BILLING_MODEL_READINESS_PLANMODE_PROMPT.md</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md</t>
+          <t>ACCOUNT_AND_BILLING_MODEL_READINESS_PLAN.md</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1231,27 +1231,93 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Scherp de samenhang tussen ExitScan, RetentieScan en toekomstige producten aan.</t>
+          <t>Aanbevolen prioriteit: Later. Beslis eerst account-, plan- en billinglogica voordat Stripe of self-service billing wordt gebouwd.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>OPS_AND_DELIVERY_SYSTEM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>OPS_AND_DELIVERY_SYSTEM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Stroomlijn delivery van sales handoff tot rapportoplevering en nazorg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerciële bewijsvoering na echte pilots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLANMODE_PROMPT.md</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Aanbevolen prioriteit: Later. Scherp de samenhang tussen ExitScan, RetentieScan en toekomstige producten aan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>CONTENT_OPERATING_SYSTEM_PLANMODE_PROMPT.md</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>CONTENT_OPERATING_SYSTEM_PLAN.md</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Niet voldaan</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Niet voldaan</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>Aanbevolen prioriteit: Later. Laat site, SEO, cases en thought leadership pas als systeem groeien na product- en funnelstabiliteit.</t>
         </is>

</xml_diff>

<commit_message>
Implement pricing and packaging source of truth
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -962,12 +962,20 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Werk prijslogica, Baseline/Live en packaging commercieel strak uit.</t>
+          <t>PRICING_AND_PACKAGING_PROGRAM_PLAN.md toegevoegd; publieke pricinglaag herschikt naar eerste trajecten, vervolgvormen, add-ons en combinatieroute. Salesdocs, proposal spines, acceptance checklist en paritytests daarop gealigneerd. Validatie bevestigd via pytest, vitest, eslint en next build.</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Repo-uitvoering afgerond op 2026-04-15</t>
         </is>
       </c>
     </row>
@@ -984,12 +992,20 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Bouw sterke voorbeeldrapporten, demo-output en showcase-assets.</t>
+          <t>SAMPLE_OUTPUT_AND_SHOWCASE_PLAN.md toegevoegd en uitgevoerd; buyer-facing sample asset registry, sample output mode, publieke pdf-mirrors, product/pricing/trust showcase-ingangen, docs/prompts en paritytests bijgewerkt.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; nog niet gepusht.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tighten live verification checklist rules
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -447,7 +447,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Live/Gepusht</t>
+          <t>Repo/Main/Deploy/Live</t>
         </is>
       </c>
     </row>
@@ -479,7 +479,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Live via main</t>
+          <t>Naar main gepusht op 2026-04-14; live-status historisch niet apart vastgelegd in checklist.</t>
         </is>
       </c>
     </row>
@@ -511,7 +511,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Live op main; Supabase RPC toegepast en kernfixes hergevalideerd.</t>
+          <t>Live bevestigd op 2026-04-14; kernfixes hergevalideerd op live flow na deploy op main.</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Live via main</t>
+          <t>Naar main gepusht op 2026-04-14; live-status historisch niet apart vastgelegd in checklist.</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Voldaan; repo- en livewijzigingen doorgevoerd op main. Externe ops-note: Resend-domeinverificatie nog open voor maillevering.</t>
+          <t>Live bevestigd op 2026-04-14; repo- en livewijzigingen doorgevoerd. Externe ops-note: Resend-domeinverificatie nog open voor maillevering.</t>
         </is>
       </c>
     </row>
@@ -603,7 +603,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Live via main</t>
+          <t>Naar main gepusht op 2026-04-14; live-status historisch niet apart vastgelegd in checklist.</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Live via main</t>
+          <t>Naar main gepusht op 2026-04-14; live-status historisch niet apart vastgelegd in checklist.</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; backend- en frontend-validatie groen.</t>
+          <t>Naar main gepusht op 2026-04-14; live-status niet apart geverifieerd. Backend- en frontend-validatie groen.</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Live via main</t>
+          <t>Naar main gepusht op 2026-04-14; live-status historisch niet apart vastgelegd in checklist.</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Live via main</t>
+          <t>Naar main gepusht op 2026-04-14; live-status historisch niet apart vastgelegd in checklist.</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Naar main gepusht op 2026-04-14 (commit 7025245).</t>
+          <t>Naar main gepusht op 2026-04-14 (commit 7025245); live-status niet apart geverifieerd.</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; gepusht naar main op 2026-04-14.</t>
+          <t>Naar main gepusht op 2026-04-14; live-status niet apart geverifieerd.</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo en live bevestigd; frontend tests, lint, build, backend paritytests en productie smoke checks groen bevestigd.</t>
+          <t>Live bevestigd op 2026-04-15; frontend tests, lint, build, backend paritytests en productie smoke checks groen bevestigd.</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ja: live bevestigd op 2026-04-15 via https://www.verisight.nl, /tarieven en /vertrouwen; founder-led termen zichtbaar.</t>
+          <t>Live bevestigd op 2026-04-15 via https://www.verisight.nl, /tarieven en /vertrouwen; founder-led termen zichtbaar.</t>
         </is>
       </c>
     </row>
@@ -915,7 +915,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Live via main</t>
+          <t>Naar main gepusht op 2026-04-15; live-status niet apart geverifieerd.</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1005,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo; nog niet gepusht.</t>
+          <t>Naar main gepusht op 2026-04-15; live-status niet lokaal geverifieerd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement website redesign and flow plan
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1022,12 +1022,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Doe website-redesign pas na trust, actionability, packaging en sample output.</t>
+          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md toegevoegd; publieke marketinglaag herbouwd voor homepage, productenoverzicht, productdetail, aanpak en tarieven. Shared content, CTA-hierarchie, preview/showcase-proof en visuele ritmiek aangescherpt; marketing-flow test toegevoegd; tests, lint, build en code-level parity checks groen.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo; naar main gepusht in deze tranche.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Strengthen visible website redesign hero pass
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1032,12 +1032,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md toegevoegd; publieke marketinglaag herbouwd voor homepage, productenoverzicht, productdetail, aanpak en tarieven. Shared content, CTA-hierarchie, preview/showcase-proof en visuele ritmiek aangescherpt; marketing-flow test toegevoegd; tests, lint, build en code-level parity checks groen.</t>
+          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md toegevoegd en verder aangescherpt; publieke marketinglaag herbouwd voor homepage, productenoverzicht, productdetail, aanpak en tarieven. Daarna tweede zichtbare visual pass uitgevoerd op homepage en producthero's met donker stage-contrast, sterkere asymmetrie en minder catalogusgevoel. Tests, lint, build en code-level parity checks groen.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Naar main gepusht op 2026-04-15; live-status niet apart geverifieerd.</t>
+          <t>Naar main gepusht op 2026-04-15; live-status na tweede visual pass nog te verifi?ren.</t>
         </is>
       </c>
     </row>
@@ -1054,12 +1054,20 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Stem funnel en klantreis af nadat website- en packagingrichting scherper staan.</t>
+          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLAN.md toegevoegd als source of truth; route-aware CTA-flow, uitgebreide contactcontracten, buyer-facing handoff-copy, salesdoc-alignment en regressietests voor funnelcontext zijn in repo doorgevoerd.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Repo bijgewerkt op 2026-04-15; nog niet naar main gepusht of live gedeployed in deze thread.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update funnel checklist live status
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1062,12 +1062,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLAN.md toegevoegd als source of truth; route-aware CTA-flow, uitgebreide contactcontracten, buyer-facing handoff-copy, salesdoc-alignment en regressietests voor funnelcontext zijn in repo doorgevoerd.</t>
+          <t>CUSTOMER_JOURNEY_AND_FUNNEL_ALIGNMENT_PLAN.md uitgevoerd; route-aware CTA-flow, uitgebreide contactcontracten, buyer-facing handoff-copy, salesdoc-alignment, acceptance-checklist en regressietests zijn doorgevoerd en lokaal gevalideerd.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Repo bijgewerkt op 2026-04-15; nog niet naar main gepusht of live gedeployed in deze thread.</t>
+          <t>Naar main gepusht en live bevestigd op 2026-04-15. Vercel production deployment dpl_J3oMQDbCmqAwWc5xwXtBP3qNb6cx staat op commit dc285c72ae4dc7e5705ffd62c730e494870500f2; www.verisight.nl en /producten/retentiescan geven de nieuwe funnelcopy en route-aware CTA-hrefs terug.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement SEO conversion program tranche
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1084,12 +1084,20 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Daarna. Optimaliseer SEO en conversie pas na website-redesign en stabiele messaging.</t>
+          <t>SEO_CONVERSION_PROGRAM_PLAN.md toegevoegd; compacte SEO-conversietranche uitgevoerd met nieuwe /oplossingen-landingspagina's, inline route-aware formulieren op money pages, metadata/sitemap/llms-alignment, pdf noindex-headers en regressietests. Validatie bevestigd via vitest, eslint en next build.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo op 2026-04-15; nog niet gepusht of live geverifieerd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record live visual integrity verification
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1032,12 +1032,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md toegevoegd en verder aangescherpt; publieke marketinglaag herbouwd voor homepage, productenoverzicht, productdetail, aanpak en tarieven. Daarna tweede zichtbare visual pass uitgevoerd op homepage en producthero's met donker stage-contrast, sterkere asymmetrie en minder catalogusgevoel. Tests, lint, build en code-level parity checks groen.</t>
+          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md toegevoegd en aangescherpt; publieke marketinglaag eerder herbouwd. Daarna gerichte visual integrity pass uitgevoerd op homepage, productenoverzicht en gedeelde hero-shell: kolombreedtes, headline-measures, CTA-rijen, stage-balans en breakpoint-QA aangescherpt. Lint, tests, build en browsermatige screenshot-QA uitgevoerd.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Naar main gepusht op 2026-04-15; live-status na tweede visual pass nog te verifi?ren.</t>
+          <t>Live bevestigd op 2026-04-15 via productie-URL's; visuele integriteitspass per breakpoint gecontroleerd; commit 4ef87d1.</t>
         </is>
       </c>
     </row>
@@ -1114,12 +1114,20 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Richt onboarding, livegang en eerste managementgebruik beter in zodra commerciële basis staat.</t>
+          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLAN.md blijft source of truth; buyer-facing handoff, admin onboardingblueprint, setup/importverwachtingen, klantactivatie, dashboard- en campaignadoptie, ops-playbook, acceptance-checklist en regressietests zijn nu daadwerkelijk in repo doorgevoerd.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo op 2026-04-15; docs, frontend flows en tests bijgewerkt. Niet naar main gepusht en niet live gedeployed in deze tranche.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement client onboarding and adoption layer
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1122,12 +1122,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLAN.md blijft source of truth; buyer-facing handoff, admin onboardingblueprint, setup/importverwachtingen, klantactivatie, dashboard- en campaignadoptie, ops-playbook, acceptance-checklist en regressietests zijn nu daadwerkelijk in repo doorgevoerd.</t>
+          <t>CLIENT_ONBOARDING_AND_ADOPTION_PROGRAM_PLAN.md blijft source of truth; buyer-facing handoff, admin onboardingblueprint, setup/importverwachtingen, klantactivatie, dashboard- en campaignadoptie, ops-playbook, acceptance-checklist, regressietests en lokale flowchecks zijn nu daadwerkelijk in repo doorgevoerd.</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo op 2026-04-15; docs, frontend flows en tests bijgewerkt. Niet naar main gepusht en niet live gedeployed in deze tranche.</t>
+          <t>Uitgevoerd in repo op 2026-04-15; docs, frontend flows en tests bijgewerkt. Frontend test/lint/build groen en lokale routechecks uitgevoerd. Niet eerder gepusht; deze commit brengt de tranche naar main.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document broad visual integrity repair
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1032,12 +1032,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md toegevoegd en aangescherpt; publieke marketinglaag eerder herbouwd. Daarna gerichte visual integrity pass uitgevoerd op homepage, productenoverzicht en gedeelde hero-shell: kolombreedtes, headline-measures, CTA-rijen, stage-balans en breakpoint-QA aangescherpt. Lint, tests, build en browsermatige screenshot-QA uitgevoerd.</t>
+          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md uitgevoerd en daarna breder hersteld met een whole-site visual integrity pass. Gedeelde marketing-shell aangescherpt op hero-opbouw, stage-volgorde, supportvolgorde, type scale, header-breakpoints en tabletnavigatie. Lint, tests, build en browsermatige screenshot-QA op desktop, tablet en mobiel uitgevoerd.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Live bevestigd op 2026-04-15 via productie-URL's; visuele integriteitspass per breakpoint gecontroleerd; visual-pass commit 4ef87d1; checklist bevestigd in commit bdb653f.</t>
+          <t>Live bevestigd op 2026-04-15 via productie-URL's; brede visual integrity pass per breakpoint gecontroleerd; commit 738b8f0.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement implementation readiness workflow
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1144,12 +1144,15 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Maak implementation readiness schaalbaar na scherpere commerciële en websitebasis.</t>
+          <t>Planbestand gemaakt, implementation readiness uitgevoerd, validatie gedraaid en docs/checklists toegevoegd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify implementation readiness release status
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1155,6 +1155,11 @@
           <t>Planbestand gemaakt, implementation readiness uitgevoerd, validatie gedraaid en docs/checklists toegevoegd.</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Naar main gepusht op 2026-04-15 (41936db); live-status niet lokaal geverifieerd.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Document marketing UI stabilization pass
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1032,12 +1032,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md uitgevoerd en daarna breder hersteld met een whole-site visual integrity pass. Gedeelde marketing-shell aangescherpt op hero-opbouw, stage-volgorde, supportvolgorde, type scale, header-breakpoints en tabletnavigatie. Lint, tests, build en browsermatige screenshot-QA op desktop, tablet en mobiel uitgevoerd.</t>
+          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md uitgevoerd en daarna verbreed met een marketing UI stabilization pass. Gedeelde shell aangescherpt op hero-opbouw, stage-volgorde, supportvolgorde, type scale, header-breakpoints, flow-stack en compactere preview/proof-rails. Lint, tests, build en browsermatige screenshot-QA op desktop, tablet en mobiel uitgevoerd.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Live bevestigd op 2026-04-15 via productie-URL's; brede visual integrity pass per breakpoint gecontroleerd; commit 738b8f0.</t>
+          <t>Live bevestigd op 2026-04-15 via productie-URL's; marketing UI stabilization pass per breakpoint gecontroleerd; commit 37cbf6e.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add pilot and early customer learning system
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1206,12 +1206,22 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Borg leerloops en pilotfeedback zodra eerste klanttrajecten lopen.</t>
+          <t>PILOT_AND_EARLY_CUSTOMER_LEARNING_SYSTEM_PLAN.md toegevoegd; persisted learningdossiers en checkpoints ingebouwd in backend/supabase, admin-workbench toegevoegd, ops-playbook/templates toegevoegd en gevalideerd met pytest, vitest, lint en build.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Repo lokaal uitgevoerd en gevalideerd op 2026-04-15; main/deploy/live zijn in deze thread niet uitgevoerd.</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1238,20 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Maak demo-omgeving en voorbeeldcampagnes schaalbaar na sample-output en salesbasis.</t>
+          <t>docs/active/DEMO_AND_SAMPLE_ENVIRONMENT_PROGRAM_PLAN.md toegevoegd en uitgevoerd; canonieke demo-laagindeling, demo_environment.py, manage_demo_environment.py, demo system/playbook/acceptance docs, promptverwijzingen en regressietests bijgewerkt.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Uitgevoerd in repo op 2026-04-15; py_compile en manage_demo_environment list groen, python -m pytest tests/test_demo_environment_system.py tests/test_sample_generator.py -q groen.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document live page-type composition verification
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1032,12 +1032,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md uitgevoerd en daarna verbreed met een marketing UI stabilization pass. Gedeelde shell aangescherpt op hero-opbouw, stage-volgorde, supportvolgorde, type scale, header-breakpoints, flow-stack en compactere preview/proof-rails. Lint, tests, build en browsermatige screenshot-QA op desktop, tablet en mobiel uitgevoerd.</t>
+          <t>WEBSITE_REDESIGN_AND_FLOW_PLAN.md uitgevoerd en daarna verbreed met een marketing UI stabilization pass en een gecontroleerde compositiepass per paginatype. Gedeelde shell aangescherpt op page-type hero-compositie, title-scales, stage-title-scales, supportgewicht, hero-grid-verhoudingen en vervolglinks. Lint, tests, build en browsermatige screenshot-QA lokaal en live uitgevoerd op desktop, tablet en mobiel.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Live bevestigd op 2026-04-15 via productie-URL's; marketing UI stabilization pass per breakpoint gecontroleerd; commit 37cbf6e.</t>
+          <t>Live bevestigd op 2026-04-15 via productie-URL's; visuele integriteitspass per breakpoint gecontroleerd; compositiepass per paginatype live bevestigd op desktop, tablet en mobiel; commit 4d044c6.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record live status for pilot learning tranche
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1216,12 +1216,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PILOT_AND_EARLY_CUSTOMER_LEARNING_SYSTEM_PLAN.md toegevoegd; persisted learningdossiers en checkpoints ingebouwd in backend/supabase, admin-workbench toegevoegd, ops-playbook/templates toegevoegd en gevalideerd met pytest, vitest, lint en build.</t>
+          <t>PILOT_AND_EARLY_CUSTOMER_LEARNING_SYSTEM_PLAN.md toegevoegd; persisted learningdossiers en checkpoints ingebouwd, admin-workbench toegevoegd, ops-playbook/templates toegevoegd en gevalideerd met pytest, vitest, lint en build. Live-status daarna bevestigd op het gekoppelde Vercel-project.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Repo lokaal uitgevoerd en gevalideerd op 2026-04-15; main/deploy/live zijn in deze thread niet uitgevoerd.</t>
+          <t>Naar main gepusht op 2026-04-15; live bevestigd via Vercel production deployment op main met aliassen verisight.nl en verisight-saa-s.vercel.app.</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo op 2026-04-15; py_compile en manage_demo_environment list groen, python -m pytest tests/test_demo_environment_system.py tests/test_sample_generator.py -q groen.</t>
+          <t>Uitgevoerd in repo op 2026-04-15; py_compile en manage_demo_environment list groen, python -m pytest tests/test_demo_environment_system.py tests/test_sample_generator.py -q groen. Publieke site https://www.verisight.nl is live bereikbaar en toont de sample/showcase-laag; Vercel deploymentmetadata kon hier niet direct geverifieerd worden omdat auth vereist is.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add assisted-to-SaaS readiness plan
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1268,12 +1268,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Bepaal wanneer en hoe Verisight van assisted/productized aanbod richting SaaS-readiness mag bewegen.</t>
+          <t>ASSISTED_TO_SAAS_READINESS_PROGRAM_PLAN.md toegevoegd als actieve source of truth; assisted, semi-self-service, readiness-gates en false-SaaS guardrails repo-gebaseerd vastgelegd.</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Repo-only bevestigd op 2026-04-15; docs/active-plan toegevoegd, checklist bijgewerkt en roadmap gesynchroniseerd. Geen deploy of live-wijziging in deze tranche.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement customer lifecycle and expansion model
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1300,12 +1300,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Werk de route uit van eerste sale naar herhaalgebruik, uitbreiding en productdoorstroom.</t>
+          <t>CUSTOMER_LIFECYCLE_AND_EXPANSION_MODEL_PLAN.md blijft source of truth; lifecycle-ladder, buyer-facing pricing/aanpak/contactcopy, in-product vervolgkeuzes, pilot-learning capture, regressietests, build en roadmap-sync zijn nu daadwerkelijk in repo doorgevoerd.</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Repo uitgevoerd op 2026-04-15; actieve source of truth in docs/active/CUSTOMER_LIFECYCLE_AND_EXPANSION_MODEL_PLAN.md; frontend test/lint/build groen; geen push/live stap bevestigd in checkliststatus zelf.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record live status for lifecycle expansion tranche
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1310,12 +1310,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CUSTOMER_LIFECYCLE_AND_EXPANSION_MODEL_PLAN.md blijft source of truth; lifecycle-ladder, buyer-facing pricing/aanpak/contactcopy, in-product vervolgkeuzes, pilot-learning capture, regressietests, build en roadmap-sync zijn nu daadwerkelijk in repo doorgevoerd.</t>
+          <t>CUSTOMER_LIFECYCLE_AND_EXPANSION_MODEL_PLAN.md blijft source of truth; lifecycle-ladder, buyer-facing pricing/aanpak/contactcopy, in-product vervolgkeuzes, pilot-learning capture, regressietests, build en roadmap-sync zijn in repo doorgevoerd. Live-status op 2026-04-15 geverifieerd via Vercel en productiedomeinen.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Repo uitgevoerd op 2026-04-15; actieve source of truth in docs/active/CUSTOMER_LIFECYCLE_AND_EXPANSION_MODEL_PLAN.md; frontend test/lint/build groen; geen push/live stap bevestigd in checkliststatus zelf.</t>
+          <t>Live per 2026-04-15: production deployment dpl_24rDFsoas3jfWMVD4xRvB8S2AeaR voor commit 1a0f97e04f31be272a5612278765d866664ac9d1 staat op READY. https://www.verisight.nl geeft 200 OK; https://verisight.nl redirect met 307 naar https://www.verisight.nl/.</t>
         </is>
       </c>
     </row>
@@ -1332,12 +1332,20 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Beslis eerst account-, plan- en billinglogica voordat Stripe of self-service billing wordt gebouwd.</t>
+          <t>ACCOUNT_AND_BILLING_MODEL_READINESS_PLAN.md toegevoegd als actieve source of truth; tenant/accountgrens, package- en billinggrenzen, assisted provisioningcontracten, billing-readiness gates en no-go rules repo-gebaseerd vastgelegd.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Repo-only bevestigd op 2026-04-15: docs/active-plan, checklistupdate en roadmap-sync doorgevoerd. Geen aparte livewijziging of runtime-implementatie in deze tranche.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add account and billing readiness model guards
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1335,17 +1335,19 @@
           <t>Voldaan</t>
         </is>
       </c>
-      <c r="D30" s="1" t="n">
-        <v>46127</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ACCOUNT_AND_BILLING_MODEL_READINESS_PLAN.md toegevoegd als actieve source of truth; tenant/accountgrens, package- en billinggrenzen, assisted provisioningcontracten, billing-readiness gates en no-go rules repo-gebaseerd vastgelegd.</t>
+          <t>ACCOUNT_AND_BILLING_MODEL_READINESS_PLAN.md bevestigd als actieve source of truth; architectuur, gedeelde types, buyer-facing voorwaarden en parity checks bijgewerkt om de v1-accountgrens, assisted facturatie en seat-/usage-guardrails expliciet te maken.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Repo-only bevestigd op 2026-04-15: docs/active-plan, checklistupdate en roadmap-sync doorgevoerd. Geen aparte livewijziging of runtime-implementatie in deze tranche.</t>
+          <t>Repo bevestigd op 2026-04-15: active-plan, ARCHITECTURE, frontend types, voorwaarden, parity-test, checklistupdate en roadmap-sync doorgevoerd; pytest, lint en frontend build groen. Geen aparte livewijziging of runtime-billingimplementatie in deze tranche.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark account billing readiness as live verified
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1342,12 +1342,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>ACCOUNT_AND_BILLING_MODEL_READINESS_PLAN.md bevestigd als actieve source of truth; architectuur, gedeelde types, buyer-facing voorwaarden en parity checks bijgewerkt om de v1-accountgrens, assisted facturatie en seat-/usage-guardrails expliciet te maken.</t>
+          <t>ACCOUNT_AND_BILLING_MODEL_READINESS_PLAN.md bevestigd als actieve source of truth; architectuur, gedeelde types, buyer-facing voorwaarden en parity checks bijgewerkt om de v1-accountgrens, assisted facturatie en seat-/usage-guardrails expliciet te maken. Publieke voorwaardenpagina live geverifieerd op 2026-04-15.</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Repo bevestigd op 2026-04-15: active-plan, ARCHITECTURE, frontend types, voorwaarden, parity-test, checklistupdate en roadmap-sync doorgevoerd; pytest, lint en frontend build groen. Geen aparte livewijziging of runtime-billingimplementatie in deze tranche.</t>
+          <t>Live bevestigd op 2026-04-15: active-plan, ARCHITECTURE, frontend types, voorwaarden, parity-test, checklistupdate en roadmap-sync doorgevoerd; pytest, lint en frontend build groen. Publieke productiepagina https://www.verisight.nl/voorwaarden retourneert 200 en bevat de nieuwe assisted/manual-billing copy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement persistent ops delivery control
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1364,12 +1364,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Stroomlijn delivery van sales handoff tot rapportoplevering en nazorg.</t>
+          <t>Persistente ops- en deliverylaag geimplementeerd inclusief leadtriage, deliveryrecords, checkpoints, command-center, failure matrix en campaign delivery control. Typecheck, tests, lint, build en artifact checks groen.</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Repo bijgewerkt; main/deploy/live nog niet bevestigd.</t>
         </is>
       </c>
     </row>
@@ -1386,12 +1396,20 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Organiseer klantbewijs, cases en commerciële bewijsvoering na echte pilots.</t>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md toegevoegd als source of truth; evidence-taxonomie, case-capture, approval/playbooks, sample-proof tiering en regressietests zijn repo-breed uitgewerkt.</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Lokaal in repo uitgevoerd op 2026-04-15; nog niet naar main gepusht of live geverifieerd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement case proof and evidence system
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1374,12 +1374,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Persistente ops- en deliverylaag geimplementeerd inclusief leadtriage, deliveryrecords, checkpoints, command-center, failure matrix en campaign delivery control. Typecheck, tests, lint, build en artifact checks groen.</t>
+          <t>Persistente ops- en deliverylaag geimplementeerd inclusief leadtriage, deliveryrecords, checkpoints, command-center, failure matrix en campaign delivery control. Main bijgewerkt. Live-adminverificatie geprobeerd via lokale Chrome- en Edge-profielen, maar beide profielsessies waren niet herbruikbaar voor headless verificatie.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Repo en main bijgewerkt; deploy/live nog niet bevestigd.</t>
+          <t>Repo en main bijgewerkt; publieke site bereikbaar; live-adminverificatie geprobeerd maar niet hard bevestigd door browserprofiel-lock/sessiebeperking.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update checklist with live case proof status
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1404,12 +1404,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md toegevoegd als source of truth; evidence-taxonomie, case-capture, approval/playbooks, sample-proof tiering en regressietests zijn repo-breed uitgewerkt.</t>
+          <t>CASE_PROOF_AND_EVIDENCE_PROGRAM_PLAN.md toegevoegd als source of truth; evidence-taxonomie, case-capture, approval/playbooks, sample-proof tiering en regressietests zijn repo-breed uitgewerkt, gevalideerd, gecommit en naar main gepusht.</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Lokaal in repo uitgevoerd op 2026-04-15; nog niet naar main gepusht of live geverifieerd.</t>
+          <t>Naar main gepusht op 2026-04-15; publieke site https://www.verisight.nl gecontroleerd op 2026-04-15 en de actuele buyer-facing prooflaag is zichtbaar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark ops delivery tranche live verified
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1374,12 +1374,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Persistente ops- en deliverylaag geimplementeerd inclusief leadtriage, deliveryrecords, checkpoints, command-center, failure matrix en campaign delivery control. Main bijgewerkt. Live-adminverificatie geprobeerd via lokale Chrome- en Edge-profielen, maar beide profielsessies waren niet herbruikbaar voor headless verificatie.</t>
+          <t>Persistente ops- en deliverylaag geimplementeerd inclusief leadtriage, deliveryrecords, checkpoints, command-center, failure matrix en campaign delivery control. Main bijgewerkt. Live bevestigd via admin screenshot op https://www.verisight.nl/beheer met zichtbare Setup-pagina en adminnavigatie.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Repo en main bijgewerkt; publieke site bereikbaar; live-adminverificatie geprobeerd maar niet hard bevestigd door browserprofiel-lock/sessiebeperking.</t>
+          <t>Repo, main en live bevestigd; admin Setup zichtbaar op /beheer.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement portfolio architecture program
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1426,12 +1426,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Scherp de samenhang tussen ExitScan, RetentieScan en toekomstige producten aan.</t>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md toegevoegd als actieve source of truth; marketing productmodel, publieke portfolio-copy, structured-data-hi?rarchie, regressietests en combinatie-routeframing repo-breed aangescherpt.</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Repo-only status op 2026-04-15: actieve planfile, marketing/productsurfaces, reference memo en tests bijgewerkt; nog niet naar main gepusht of live geverifieerd in deze tranche.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mark portfolio architecture tranche live verified
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1436,12 +1436,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md toegevoegd als actieve source of truth; marketing productmodel, publieke portfolio-copy, structured-data-hi?rarchie, regressietests en combinatie-routeframing repo-breed aangescherpt.</t>
+          <t>PORTFOLIO_ARCHITECTURE_PROGRAM_PLAN.md actief gemaakt als source of truth; marketing productmodel, publieke portfolio-copy, structured-data-hierarchie, regressietests en combinatie-routeframing repo-breed aangescherpt.</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Repo-only status op 2026-04-15: actieve planfile, marketing/productsurfaces, reference memo en tests bijgewerkt; nog niet naar main gepusht of live geverifieerd in deze tranche.</t>
+          <t>Live bevestigd op 2026-04-15: production deployment dpl_9BT9wVYZ4mztTxAnroBXdvjqnZP7 voor commit 9c58ce687e0922ba3861fdaadbbdf87805c3a466 staat op READY op Vercel.</t>
         </is>
       </c>
     </row>
@@ -1458,12 +1458,20 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Niet voldaan</t>
-        </is>
+          <t>Voldaan</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>46127</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Aanbevolen prioriteit: Later. Laat site, SEO, cases en thought leadership pas als systeem groeien na product- en funnelstabiliteit.</t>
+          <t>CONTENT_OPERATING_SYSTEM_PLAN.md toegevoegd als source of truth; canonieke contentarchitectuur, content-governance, surface-ownership docs, typed registry, regressietests en prompt-fix doorgevoerd.</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Repo-only bevestigd op 2026-04-15; docs/active, docs/reference, frontend/lib registry/tests, promptfix en roadmap-sync doorgevoerd. Niet gepusht of live geverifieerd.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement content operating system tranche
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1462,16 +1462,16 @@
         </is>
       </c>
       <c r="D34" s="1" t="n">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CONTENT_OPERATING_SYSTEM_PLAN.md toegevoegd als source of truth; canonieke contentarchitectuur, content-governance, surface-ownership docs, typed registry, regressietests en prompt-fix doorgevoerd.</t>
+          <t>CONTENT_OPERATING_SYSTEM_PLAN.md toegevoegd als source of truth; canonieke contentarchitectuur, content-governance, surface-ownership docs, typed registry, regressietests en prompt-fix doorgevoerd; planfile bijgewerkt met aanvullende validatie-uitkomst.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Repo-only bevestigd op 2026-04-15; docs/active, docs/reference, frontend/lib registry/tests, promptfix en roadmap-sync doorgevoerd. Niet gepusht of live geverifieerd.</t>
+          <t>Repo-only bevestigd op 2026-04-16; docs/active, docs/reference, frontend/lib registry/tests, promptfix, lint en build groen. Bestaande marketing-flow parity-test faalt op al lopende marketingcopy-wijziging buiten deze tranche.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update content operating system checklist status
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1466,12 +1466,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CONTENT_OPERATING_SYSTEM_PLAN.md toegevoegd als source of truth; canonieke contentarchitectuur, content-governance, surface-ownership docs, typed registry, regressietests en prompt-fix doorgevoerd; planfile bijgewerkt met aanvullende validatie-uitkomst.</t>
+          <t>CONTENT_OPERATING_SYSTEM_PLAN.md toegevoegd als source of truth; canonieke contentarchitectuur, content-governance, surface-ownership docs, typed registry, regressietests en prompt-fix doorgevoerd. Daarna naar main gepusht.</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Repo-only bevestigd op 2026-04-16; docs/active, docs/reference, frontend/lib registry/tests, promptfix, lint en build groen. Bestaande marketing-flow parity-test faalt op al lopende marketingcopy-wijziging buiten deze tranche.</t>
+          <t>Naar main gepusht op 2026-04-16 (commit b962034); live-status niet geverifieerd. Vercel-verificatie blokkeerde hier op auth en deze tranche heeft geen publiek herkenbare runtimewijziging.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CEO growth operating system
</commit_message>
<xml_diff>
--- a/docs/prompts/PROMPT_CHECKLIST.xlsx
+++ b/docs/prompts/PROMPT_CHECKLIST.xlsx
@@ -1097,7 +1097,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo op 2026-04-15; nog niet gepusht of live geverifieerd.</t>
+          <t>Live bevestigd op 2026-04-16 via productie-URL's; commit 10862d9.</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo op 2026-04-15; docs, frontend flows en tests bijgewerkt. Frontend test/lint/build groen en lokale routechecks uitgevoerd. Niet eerder gepusht; deze commit brengt de tranche naar main.</t>
+          <t>Live bevestigd op 2026-04-16 via https://www.verisight.nl/aanpak en publieke buyer-facing onboarding-copy; commit 7559bdc. Authenticated dashboardflow niet apart geverifieerd.</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Uitgevoerd in repo op 2026-04-15; py_compile en manage_demo_environment list groen, python -m pytest tests/test_demo_environment_system.py tests/test_sample_generator.py -q groen. Publieke site https://www.verisight.nl is live bereikbaar en toont de sample/showcase-laag; Vercel deploymentmetadata kon hier niet direct geverifieerd worden omdat auth vereist is.</t>
+          <t>Publieke sample/showcase-routes bevestigd op 2026-04-16; deploymentmetadata niet apart geverifieerd.</t>
         </is>
       </c>
     </row>

</xml_diff>